<commit_message>
Update manuscript figures and supplements
</commit_message>
<xml_diff>
--- a/manuscript_material/source_data/Source_Data_Fig3.xlsx
+++ b/manuscript_material/source_data/Source_Data_Fig3.xlsx
@@ -431,7 +431,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>galaxy_condition_mean</t>
+          <t>galaxy_condition_mean_percent</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -452,11 +452,11 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.9544</v>
+        <v>95.44</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.8901; 0.9803; 0.9928</t>
+          <t>89.01; 98.03; 99.28</t>
         </is>
       </c>
     </row>
@@ -472,11 +472,11 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.9905</v>
+        <v>99.05</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0.9928; 0.9934; 0.9854</t>
+          <t>99.28; 99.34; 98.54</t>
         </is>
       </c>
     </row>
@@ -492,11 +492,11 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.9369</v>
+        <v>93.69</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.9176; 0.9815; 0.9116</t>
+          <t>91.76; 98.15; 91.16</t>
         </is>
       </c>
     </row>
@@ -512,11 +512,11 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.9993</v>
+        <v>99.93000000000001</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.9999; 0.9992; 0.9987</t>
+          <t>99.99; 99.92; 99.87</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>89.33329999999999</v>
+        <v>89.33</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -552,7 +552,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>88.66670000000001</v>
+        <v>88.67</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -633,7 +633,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>86.66670000000001</v>
+        <v>86.67</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>91.66670000000001</v>
+        <v>91.67</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -693,7 +693,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>84.33329999999999</v>
+        <v>84.33</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -712,7 +712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -728,15 +728,20 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>user_defined_tools_offered</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>runs_requesting_a_user_defined_tool</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>galaxy_condition_runs_with_traces</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>percent</t>
         </is>
@@ -745,7 +750,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BixBench-Verified-50</t>
+          <t>IWC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -753,20 +758,25 @@
           <t>GPT-5.5</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>100</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
       </c>
       <c r="D2" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>66.7</v>
+        <v>30</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BixBench-Verified-50</t>
+          <t>IWC</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -774,20 +784,25 @@
           <t>GPT-5.6 Sol</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>52</v>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
       </c>
       <c r="D3" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>34.7</v>
+        <v>30</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BixBench-Verified-50</t>
+          <t>IWC</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -795,20 +810,25 @@
           <t>GPT-5.6 Luna</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>59</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
       </c>
       <c r="D4" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>39.3</v>
+        <v>30</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BixBench-Verified-50</t>
+          <t>IWC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -816,14 +836,19 @@
           <t>DeepSeek V4 Pro</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>14</v>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
       </c>
       <c r="D5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>9.300000000000001</v>
+        <v>30</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -834,100 +859,229 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DeepSeek V4 Pro (Claude Code, superseded)</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>42</v>
+          <t>GPT-5.5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
       </c>
       <c r="D6" t="n">
+        <v>100</v>
+      </c>
+      <c r="E6" t="n">
         <v>150</v>
       </c>
-      <c r="E6" t="n">
-        <v>28</v>
+      <c r="F6" t="n">
+        <v>66.7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CompBioBench</t>
+          <t>BixBench-Verified-50</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>263</v>
+          <t>GPT-5.6 Sol</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
       </c>
       <c r="D7" t="n">
-        <v>298</v>
+        <v>52</v>
       </c>
       <c r="E7" t="n">
-        <v>88.3</v>
+        <v>150</v>
+      </c>
+      <c r="F7" t="n">
+        <v>34.7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CompBioBench</t>
+          <t>BixBench-Verified-50</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>GPT-5.6 Sol</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>239</v>
+          <t>GPT-5.6 Luna</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
       </c>
       <c r="D8" t="n">
-        <v>300</v>
+        <v>59</v>
       </c>
       <c r="E8" t="n">
-        <v>79.7</v>
+        <v>150</v>
+      </c>
+      <c r="F8" t="n">
+        <v>39.3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CompBioBench</t>
+          <t>BixBench-Verified-50</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>GPT-5.6 Luna</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>176</v>
+          <t>DeepSeek V4 Pro</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
       </c>
       <c r="D9" t="n">
-        <v>290</v>
+        <v>14</v>
       </c>
       <c r="E9" t="n">
-        <v>60.7</v>
+        <v>150</v>
+      </c>
+      <c r="F9" t="n">
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>BixBench-Verified-50</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 Pro (Claude Code, superseded)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>42</v>
+      </c>
+      <c r="E10" t="n">
+        <v>150</v>
+      </c>
+      <c r="F10" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>CompBioBench</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>GPT-5.5</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>263</v>
+      </c>
+      <c r="E11" t="n">
+        <v>298</v>
+      </c>
+      <c r="F11" t="n">
+        <v>88.3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CompBioBench</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>GPT-5.6 Sol</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>239</v>
+      </c>
+      <c r="E12" t="n">
+        <v>300</v>
+      </c>
+      <c r="F12" t="n">
+        <v>79.7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CompBioBench</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>GPT-5.6 Luna</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>176</v>
+      </c>
+      <c r="E13" t="n">
+        <v>290</v>
+      </c>
+      <c r="F13" t="n">
+        <v>60.7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CompBioBench</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>DeepSeek V4 Pro</t>
         </is>
       </c>
-      <c r="C10" t="n">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
         <v>130</v>
       </c>
-      <c r="D10" t="n">
+      <c r="E14" t="n">
         <v>300</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F14" t="n">
         <v>43.3</v>
       </c>
     </row>
@@ -985,7 +1139,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BixBench-Verified-50</t>
+          <t>IWC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -994,25 +1148,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>150</v>
+        <v>30</v>
       </c>
       <c r="D2" t="n">
-        <v>1.19</v>
+        <v>2.349</v>
       </c>
       <c r="E2" t="n">
-        <v>0.864</v>
+        <v>1.532</v>
       </c>
       <c r="F2" t="n">
-        <v>1.664</v>
+        <v>3.514</v>
       </c>
       <c r="G2" t="n">
-        <v>0.317</v>
+        <v>1.189</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BixBench-Verified-50</t>
+          <t>IWC</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1021,25 +1175,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>150</v>
+        <v>30</v>
       </c>
       <c r="D3" t="n">
-        <v>1.557</v>
+        <v>4.229</v>
       </c>
       <c r="E3" t="n">
-        <v>1.007</v>
+        <v>2.045</v>
       </c>
       <c r="F3" t="n">
-        <v>2.614</v>
+        <v>6.087</v>
       </c>
       <c r="G3" t="n">
-        <v>0.3</v>
+        <v>1.435</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BixBench-Verified-50</t>
+          <t>IWC</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1048,25 +1202,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>150</v>
+        <v>30</v>
       </c>
       <c r="D4" t="n">
-        <v>5.026</v>
+        <v>10.157</v>
       </c>
       <c r="E4" t="n">
-        <v>2.898</v>
+        <v>5.611</v>
       </c>
       <c r="F4" t="n">
-        <v>9.388</v>
+        <v>11.999</v>
       </c>
       <c r="G4" t="n">
-        <v>0.67</v>
+        <v>3.657</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BixBench-Verified-50</t>
+          <t>IWC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1075,19 +1229,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>150</v>
+        <v>30</v>
       </c>
       <c r="D5" t="n">
-        <v>3.523</v>
+        <v>6.343</v>
       </c>
       <c r="E5" t="n">
-        <v>2.194</v>
+        <v>3.322</v>
       </c>
       <c r="F5" t="n">
-        <v>7.468</v>
+        <v>11.739</v>
       </c>
       <c r="G5" t="n">
-        <v>1.102</v>
+        <v>2.077</v>
       </c>
     </row>
     <row r="6">
@@ -1098,137 +1252,137 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DeepSeek V4 Pro (Claude Code, superseded)</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>150</v>
       </c>
       <c r="D6" t="n">
-        <v>2.068</v>
+        <v>1.19</v>
       </c>
       <c r="E6" t="n">
-        <v>1.314</v>
+        <v>0.864</v>
       </c>
       <c r="F6" t="n">
-        <v>2.898</v>
+        <v>1.664</v>
       </c>
       <c r="G6" t="n">
-        <v>0.703</v>
+        <v>0.317</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CompBioBench</t>
+          <t>BixBench-Verified-50</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
+          <t>GPT-5.6 Sol</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>297</v>
+        <v>150</v>
       </c>
       <c r="D7" t="n">
-        <v>1.735</v>
+        <v>1.557</v>
       </c>
       <c r="E7" t="n">
-        <v>0.63</v>
+        <v>1.007</v>
       </c>
       <c r="F7" t="n">
-        <v>3.895</v>
+        <v>2.614</v>
       </c>
       <c r="G7" t="n">
-        <v>0.491</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CompBioBench</t>
+          <t>BixBench-Verified-50</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>GPT-5.6 Sol</t>
+          <t>GPT-5.6 Luna</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="D8" t="n">
-        <v>3.748</v>
+        <v>5.026</v>
       </c>
       <c r="E8" t="n">
-        <v>1.438</v>
+        <v>2.898</v>
       </c>
       <c r="F8" t="n">
-        <v>10.356</v>
+        <v>9.388</v>
       </c>
       <c r="G8" t="n">
-        <v>0.531</v>
+        <v>0.67</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CompBioBench</t>
+          <t>BixBench-Verified-50</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>GPT-5.6 Luna</t>
+          <t>DeepSeek V4 Pro (Codex)</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>290</v>
+        <v>150</v>
       </c>
       <c r="D9" t="n">
-        <v>10.238</v>
+        <v>3.523</v>
       </c>
       <c r="E9" t="n">
-        <v>3.806</v>
+        <v>2.194</v>
       </c>
       <c r="F9" t="n">
-        <v>20.046</v>
+        <v>7.468</v>
       </c>
       <c r="G9" t="n">
-        <v>1.449</v>
+        <v>1.102</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CompBioBench</t>
+          <t>BixBench-Verified-50</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DeepSeek V4 Pro (Codex)</t>
+          <t>DeepSeek V4 Pro (Claude Code, superseded)</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="D10" t="n">
-        <v>8.478999999999999</v>
+        <v>2.068</v>
       </c>
       <c r="E10" t="n">
-        <v>3.58</v>
+        <v>1.314</v>
       </c>
       <c r="F10" t="n">
-        <v>20.015</v>
+        <v>2.898</v>
       </c>
       <c r="G10" t="n">
-        <v>2.408</v>
+        <v>0.703</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>IWC</t>
+          <t>CompBioBench</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1237,25 +1391,25 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>30</v>
+        <v>297</v>
       </c>
       <c r="D11" t="n">
-        <v>2.349</v>
+        <v>1.735</v>
       </c>
       <c r="E11" t="n">
-        <v>1.532</v>
+        <v>0.63</v>
       </c>
       <c r="F11" t="n">
-        <v>3.514</v>
+        <v>3.895</v>
       </c>
       <c r="G11" t="n">
-        <v>1.189</v>
+        <v>0.491</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>IWC</t>
+          <t>CompBioBench</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1264,25 +1418,25 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>30</v>
+        <v>300</v>
       </c>
       <c r="D12" t="n">
-        <v>4.229</v>
+        <v>3.748</v>
       </c>
       <c r="E12" t="n">
-        <v>2.045</v>
+        <v>1.438</v>
       </c>
       <c r="F12" t="n">
-        <v>6.087</v>
+        <v>10.356</v>
       </c>
       <c r="G12" t="n">
-        <v>1.435</v>
+        <v>0.531</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>IWC</t>
+          <t>CompBioBench</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1291,25 +1445,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>30</v>
+        <v>290</v>
       </c>
       <c r="D13" t="n">
-        <v>10.157</v>
+        <v>10.238</v>
       </c>
       <c r="E13" t="n">
-        <v>5.611</v>
+        <v>3.806</v>
       </c>
       <c r="F13" t="n">
-        <v>11.999</v>
+        <v>20.046</v>
       </c>
       <c r="G13" t="n">
-        <v>3.657</v>
+        <v>1.449</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>IWC</t>
+          <t>CompBioBench</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1318,19 +1472,19 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>30</v>
+        <v>300</v>
       </c>
       <c r="D14" t="n">
-        <v>6.343</v>
+        <v>8.478999999999999</v>
       </c>
       <c r="E14" t="n">
-        <v>3.322</v>
+        <v>3.58</v>
       </c>
       <c r="F14" t="n">
-        <v>11.739</v>
+        <v>20.015</v>
       </c>
       <c r="G14" t="n">
-        <v>2.077</v>
+        <v>2.408</v>
       </c>
     </row>
   </sheetData>

</xml_diff>